<commit_message>
Add fieldwork team planner to Sample Size Calculator (web + Excel)
- New section below sample size results: enumerator/supervisor planning
  with interviews/day, travel days, teams, training, buffer
- Auto-linked to sample size output for live recalculation
- New Fieldwork Planning tab in Excel with formulas linked to sample size
- Updated download button text and file tree description
- Added 25-30 cluster rationale note to parameter explainer

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/projects/mortality-toolkit/downloads/Sample_Size_Calculator.xlsx
+++ b/projects/mortality-toolkit/downloads/Sample_Size_Calculator.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample Size Calculator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fieldwork Planning" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,8 +78,14 @@
       <color rgb="00166534"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0078716C"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +108,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
         <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F4"/>
+        <bgColor rgb="00F5F5F4"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -146,6 +160,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -803,4 +820,438 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000369A1"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FIELDWORK TEAM PLANNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Converts sample size into enumerator teams, supervisors, and fieldwork duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>PARAMETER</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>VALUE</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>GUIDANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Interviews per enumerator per day</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Mortality surveys: 4-6/day. Depends on terrain, density, interview length (~30-45 min).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Travel days between clusters</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0.5 if close; 1-2 in dispersed, conflict-affected or mountainous settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Enumerators per team</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>4-6 per team. Larger teams finish faster but harder to supervise and transport.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Supervisor ratio (enum per supervisor)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>1 supervisor per 4-6 enumerators. Supervisors run quality checks and community entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Number of field teams</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>More teams = shorter fieldwork, higher cost. 2-3 teams is typical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Training days</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>3 days for enumerator training. Add 1-2 days for pilot testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Buffer days (weather, access, rest)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Rain, road closures, security incidents, rest days. 1-3 depending on context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>LINKED FROM SAMPLE SIZE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Number of clusters</t>
+        </is>
+      </c>
+      <c r="B15" s="15">
+        <f>'Sample Size Calculator'!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Households per cluster</t>
+        </is>
+      </c>
+      <c r="B16" s="15">
+        <f>'Sample Size Calculator'!B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Total households</t>
+        </is>
+      </c>
+      <c r="B17" s="15">
+        <f>'Sample Size Calculator'!B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>FIELDWORK CALCULATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Data collection days per cluster</t>
+        </is>
+      </c>
+      <c r="B21" s="9">
+        <f>ROUNDUP(B16/(B7*B5),0)</f>
+        <v/>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>HH per cluster / (enumerators x interviews/day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Clusters per team</t>
+        </is>
+      </c>
+      <c r="B22" s="9">
+        <f>ROUNDUP(B15/B9,0)</f>
+        <v/>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Total clusters / number of teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Field days per team</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>B21*B22+B6*(B22-1)</f>
+        <v/>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Collection days + travel between clusters</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Total enumerators</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>B7*B9</f>
+        <v/>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Enumerators per team x teams</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Supervisors needed</t>
+        </is>
+      </c>
+      <c r="B25" s="9">
+        <f>ROUNDUP(B24/B8,0)</f>
+        <v/>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Total enumerators / supervisor ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Total field staff</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>B24+B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Enumerators + supervisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Data collection duration (days)</t>
+        </is>
+      </c>
+      <c r="B28" s="9">
+        <f>B23</f>
+        <v/>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Longest team determines duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
+        <f>B10</f>
+        <v/>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>B11</f>
+        <v/>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL FIELDWORK DURATION (days)</t>
+        </is>
+      </c>
+      <c r="B31" s="12">
+        <f>B28+B29+B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Approximate weeks</t>
+        </is>
+      </c>
+      <c r="B32" s="16">
+        <f>ROUNDUP(B31/7,1)</f>
+        <v/>
+      </c>
+      <c r="C32" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>LOGISTICS CHECKLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Vehicles: 1 per team (with drivers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Tablets/phones: 1 per enumerator, loaded with XLSForm</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Supervisor kits: daily data quality checklists, cluster maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Enumerator kits: ID badge, consent forms, referral cards, pens</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Per diem: all field staff x field days</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Fuel and vehicle maintenance budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Communication: airtime for all field staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>[ ]  Data backup: portable power banks, Wi-Fi/cellular coverage plan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>